<commit_message>
Refine manuscript availability and troubleshooting updates
</commit_message>
<xml_diff>
--- a/paper/supplementary/Supplementary_Data_1.xlsx
+++ b/paper/supplementary/Supplementary_Data_1.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -60,9 +68,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,57 +437,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Supplementary Data 1</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source data for Supplementary Figures and reviewer-relevant benchmark tables in the DELT-Hit Nature Protocols supplementary notes.</t>
+          <t>Source data for the Supplementary Figures and supplementary comparison and benchmark tables.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Generated by</t>
+          <t>Supporting-material repository</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>paper/supplementary/build_submission_assets.py</t>
+          <t>https://doi.org/10.6084/m9.figshare.31198468</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NF2 rank source</t>
+          <t>DELT-Hit Zenodo archive</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/home/leandro/projects/overleaf-delt-hit-review/supporting_material/experiments/favalli/benchmark_nf2/strict14_method_ranks.csv</t>
+          <t>https://doi.org/10.5281/zenodo.20447074</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Demultiplex source</t>
+          <t>example-single-stranded: Figshare article API</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/home/leandro/projects/overleaf-delt-hit-review/benchmarks/demultiplex/tools</t>
+          <t>https://api.figshare.com/v2/articles/31198468</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>example-single-stranded: campaign.fastq.gz</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://figshare.com/ndownloader/files/61487743</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>favalli: lane-1 FASTA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/9xZkcW5jWtLHiFo/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>favalli: published evaluation table</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/cgxBWkHnpkT6rBi/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pure-del: lane-1 FASTQ</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/H8YB6wdxpwWgzLB/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pure-del: lane-2 FASTQ</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/wK6t8qjDTay8rAg/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>pure-del: published selection tables ZIP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://zenodo.org/records/11122901/files/Keller_Petrov_etal_Supplementary_Material2_Sequencing_Data.zip?download=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Generated by</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>manual README refresh; full workbook generator currently references removed NF2 assets</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6196,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6117,7 +6208,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6130,7 +6220,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6138,7 +6227,6 @@
           <t>Single-compound structure lookup</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>yes</t>
@@ -6156,7 +6244,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update supplementary links and analysis wording
</commit_message>
<xml_diff>
--- a/paper/supplementary/Supplementary_Data_1.xlsx
+++ b/paper/supplementary/Supplementary_Data_1.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,77 +445,101 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Supporting-material repository</t>
+          <t>Workflow data archive (Zenodo)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://doi.org/10.6084/m9.figshare.31198468</t>
+          <t>https://doi.org/10.5281/zenodo.20447074</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Example single-stranded direct download</t>
+          <t>Code release archive (Zenodo)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://figshare.com/ndownloader/files/61487743</t>
+          <t>https://doi.org/10.5281/zenodo.20497548</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Download links used by supporting_material/experiments/*/download.sh</t>
+          <t>Supporting-material repository</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.6084/m9.figshare.31198468</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>example-single-stranded/download.sh</t>
+          <t>Example single-stranded direct download</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://api.figshare.com/v2/articles/31198468 ; https://figshare.com/ndownloader/files/61487743</t>
+          <t>https://ndownloader.figshare.com/files/61487743</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>favalli/download.sh</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>https://polybox.ethz.ch/index.php/s/9xZkcW5jWtLHiFo/download ; https://polybox.ethz.ch/index.php/s/cgxBWkHnpkT6rBi/download</t>
+          <t>Download links used by supporting_material/experiments/*/download.sh</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>pure-del/download.sh</t>
+          <t>example-single-stranded/download.sh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://polybox.ethz.ch/index.php/s/H8YB6wdxpwWgzLB/download ; https://polybox.ethz.ch/index.php/s/wK6t8qjDTay8rAg/download ; https://zenodo.org/records/11122901/files/Keller_Petrov_etal_Supplementary_Material2_Sequencing_Data.zip?download=1</t>
+          <t>https://api.figshare.com/v2/articles/31198468 ; https://ndownloader.figshare.com/files/61487743</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>favalli/download.sh</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/9xZkcW5jWtLHiFo/download ; https://polybox.ethz.ch/index.php/s/cgxBWkHnpkT6rBi/download</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pure-del/download.sh</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://polybox.ethz.ch/index.php/s/H8YB6wdxpwWgzLB/download ; https://polybox.ethz.ch/index.php/s/wK6t8qjDTay8rAg/download ; https://zenodo.org/records/11122901/files/Keller_Petrov_etal_Supplementary_Material2_Sequencing_Data.zip?download=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Generated by</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>paper/supplementary/build_submission_assets.py</t>
         </is>

</xml_diff>

<commit_message>
Clarify timing assumptions for library complexity
</commit_message>
<xml_diff>
--- a/paper/supplementary/Supplementary_Data_1.xlsx
+++ b/paper/supplementary/Supplementary_Data_1.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SuppTable6_ReactionTemplates" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -33,7 +32,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -61,7 +63,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,7 +427,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col width="100.83203125" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -500,7 +505,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>example-single-stranded/download.sh</t>
+          <t>example-single-display/download.sh</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -557,7 +562,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1393,7 +1398,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -2229,7 +2234,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3203,7 +3208,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3414,7 +3419,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3660,7 +3665,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3809,7 +3814,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3822,7 +3826,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3835,7 +3838,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3843,7 +3845,6 @@
           <t>Single-compound structure lookup</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>yes</t>
@@ -3861,7 +3862,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3875,7 +3875,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">

</xml_diff>